<commit_message>
Changed the hard coded path in config to an excel file on the virtual machine to a storage bucket location and modifed the config strPath varialbe to be a storage bucket in orchestrator.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\narobottest\.nuget\packages\ckme-release.prices\1.0.2\content\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CKME\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62303E81-1A0A-4467-A05D-E9E28C78EDA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BC23BCE-134E-42B0-B300-DFDF62388F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="33440" windowHeight="10050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="46">
   <si>
     <t>Name</t>
   </si>
@@ -165,7 +165,13 @@
     <t>Excel.Sheet("Upload")</t>
   </si>
   <si>
-    <t>C:\Users\narobottest\.nuget\packages\ckmprp-update.standard.price.of.materials\1.0.2\content\Data\CKMPRP_Price.xlsx</t>
+    <t>CKMPRP_Price.xlsx</t>
+  </si>
+  <si>
+    <t>StorageBucketName</t>
+  </si>
+  <si>
+    <t>CKMPRP_Price</t>
   </si>
 </sst>
 </file>
@@ -562,13 +568,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:Z893"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:Z894"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="28.7265625" customWidth="1"/>
-    <col min="2" max="2" width="32.453125" customWidth="1"/>
-    <col min="3" max="3" width="81.453125" customWidth="1"/>
-    <col min="4" max="26" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1" width="24.85546875" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="81.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -617,7 +623,7 @@
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="4" spans="1:26" ht="29">
+    <row r="4" spans="1:26" ht="30">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -671,17 +677,24 @@
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A12" s="2" t="s">
+      <c r="A12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A13" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C13" s="8" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1562,6 +1575,7 @@
     <row r="891" ht="14.25" customHeight="1"/>
     <row r="892" ht="14.25" customHeight="1"/>
     <row r="893" ht="14.25" customHeight="1"/>
+    <row r="894" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1576,12 +1590,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:Z987"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.453125" customWidth="1"/>
-    <col min="4" max="26" width="8.7265625" customWidth="1"/>
+    <col min="3" max="3" width="75.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1618,7 +1632,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="29">
+    <row r="2" spans="1:26" ht="30">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2687,12 +2701,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.81640625" customWidth="1"/>
-    <col min="2" max="2" width="30.1796875" customWidth="1"/>
-    <col min="3" max="3" width="60.26953125" customWidth="1"/>
-    <col min="4" max="26" width="65.453125" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="3" max="3" width="60.28515625" customWidth="1"/>
+    <col min="4" max="26" width="65.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -3747,12 +3761,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB603F1B9C174541A09CAD297DED3959" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0e1b4b84bb3fa78649dc5ec4b1f79dba">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="96a3b727-65f7-4804-913d-e1d9b359a71e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1e7885ab2dc3e881db75b242630d58d3" ns2:_="">
     <xsd:import namespace="96a3b727-65f7-4804-913d-e1d9b359a71e"/>
@@ -3924,6 +3932,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9EA87DA7-892B-409E-AD3C-78B1CD212A0E}">
   <ds:schemaRefs>
@@ -3933,15 +3947,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E1F3F5C-7107-45F9-A38F-4418559FA17A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A00C005-442B-4AC1-B595-CAEE97B662AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3957,4 +3962,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E1F3F5C-7107-45F9-A38F-4418559FA17A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>